<commit_message>
Deployed 12e8888 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/soma.xlsx
+++ b/artifacts/soma.xlsx
@@ -1,64 +1,64 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="NamedThing" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="KeyEvent" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="KeyEventRelationship" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AdverseOutcome" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="AdverseOutcomePathway" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="MolecularInitiatingEvent" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="StudySubject" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ModelSystem" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="InVivoSubject" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="PopulationSubject" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Protocol" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ImagingProtocol" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="StainingProtocol" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="SpirometryProtocol" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="MolecularAssayProtocol" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="QuantityValue" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Unit" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="NamedEntity" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="CellTypeReference" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="SpeciesReference" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="ChemicalEntityReference" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="AnatomicalEntityReference" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="ExposureCondition" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="CellularSystem" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="CellLine" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="CellCultureConditions" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="CellCultureMedium" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="MediumSupplement" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="QuantityRange" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="CiliaryFunctionAssay" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="CiliaryFunctionOutput" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="ASLAssay" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="ASLOutput" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="MucociliaryClearanceAssay" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="MucociliaryClearanceOutput" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="OxidativeStressAssay" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="OxidativeStressOutput" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="CFTRFunctionAssay" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="CFTRFunctionOutput" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="EGFRSignalingAssay" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="EGFRSignalingOutput" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="GobletCellAssay" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="GobletCellOutput" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="BALFSputumAssay" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="BALFSputumOutput" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="LungFunctionAssay" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="LungFunctionOutput" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="FoxJExpressionAssay" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="FoxJExpressionOutput" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="GeneExpressionAssay" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="GeneExpressionOutput" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="Container" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NamedThing" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KeyEvent" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KeyEventRelationship" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdverseOutcome" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AdverseOutcomePathway" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MolecularInitiatingEvent" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StudySubject" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModelSystem" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InVivoSubject" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PopulationSubject" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ImagingProtocol" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StainingProtocol" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpirometryProtocol" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MolecularAssayProtocol" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantityValue" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NamedEntity" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellTypeReference" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SpeciesReference" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChemicalEntityReference" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnatomicalEntityReference" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ExposureCondition" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellularSystem" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellLine" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureConditions" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CellCultureMedium" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MediumSupplement" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QuantityRange" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionAssay" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CiliaryFunctionOutput" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLAssay" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASLOutput" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceAssay" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MucociliaryClearanceOutput" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressAssay" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OxidativeStressOutput" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionAssay" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CFTRFunctionOutput" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingAssay" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EGFRSignalingOutput" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellAssay" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GobletCellOutput" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumAssay" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BALFSputumOutput" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionAssay" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LungFunctionOutput" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionAssay" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FoxJExpressionOutput" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionAssay" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GeneExpressionOutput" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Container" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>